<commit_message>
chore: update allowance template with new formatting
</commit_message>
<xml_diff>
--- a/templates/allowance_template.xlsx
+++ b/templates/allowance_template.xlsx
@@ -1,38 +1,110 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25000" windowHeight="10000" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Period</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>EMP ID NO</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Name</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Department</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Total Pay</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+      </rPr>
+      <t>Email</t>
+    </r>
+  </si>
+  <si>
+    <t>DECEMBER 2025</t>
+  </si>
+  <si>
+    <r>
+      <t>MP-2026-123</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Dela Cruz, Juan Pedro</t>
+    </r>
+  </si>
+  <si>
+    <t>Production</t>
+  </si>
+  <si>
+    <r>
+      <t>juan.delacruz@example.com</t>
+    </r>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -42,6 +114,9 @@
         <fgColor rgb="00366092"/>
         <bgColor rgb="00366092"/>
       </patternFill>
+    </fill>
+    <fill>
+      <patternFill/>
     </fill>
   </fills>
   <borders count="1">
@@ -57,86 +132,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -424,82 +440,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Period</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>EMP ID NO</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Department</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Total Pay</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>DECEMBER 2025</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>MP-2022-352</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Barreda, Jeffrey Fernandez</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2">
         <v>2386.36</v>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>jeffrey.barreda@example.com</t>
-        </is>
+      <c r="F2" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>